<commit_message>
Ładowanie zdjęć schronisk do index.html
</commit_message>
<xml_diff>
--- a/Schroniska_gotowe.xlsx
+++ b/Schroniska_gotowe.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,15 +433,40 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Wysokość n.p.m.</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Lokalizacja</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Liczba dostępnych miejsc</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Ceny noclegu</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Ocena gości</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Zdjęcie</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
         <is>
           <t>lat</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>lon</t>
         </is>
@@ -456,13 +485,34 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>630 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Ustrzyki Górskie 4, 38-713</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 55 zł </t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>8,5/10</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-kremenaros.jpg</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
         <v>49.251213</v>
       </c>
-      <c r="E2" t="n">
+      <c r="J2" t="n">
         <v>22.69582</v>
       </c>
     </row>
@@ -479,14 +529,37 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>663 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t xml:space="preserve">
 82, Cisna, Polska</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 80 zł </t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>8,2/10</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Bacowka-PTTK-Pod-Honem.jpg</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
         <v>49.21433</v>
       </c>
-      <c r="E3" t="n">
+      <c r="J3" t="n">
         <v>22.31386</v>
       </c>
     </row>
@@ -503,13 +576,36 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>605 m n.p.m</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Jaworzec 1, 38-608 Wetlina</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
+        <v>24</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 85 zł </t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>9,3/10</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-Jaworzec.jpg</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
         <v>49.1583</v>
       </c>
-      <c r="E4" t="n">
+      <c r="J4" t="n">
         <v>22.4682</v>
       </c>
     </row>
@@ -526,13 +622,36 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>930 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>38-713 Brzegi Górne</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
+        <v>27</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 25 zł </t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Bacowka-PTTK-Pod-Mala-Rawka.jpg</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>49.11709</v>
       </c>
-      <c r="E5" t="n">
+      <c r="J5" t="n">
         <v>22.58094</v>
       </c>
     </row>
@@ -549,13 +668,36 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>490 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Komancza 26, Komańcza, 38-543, Polska</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
+        <v>49</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 20 zł </t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>7,9/10</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-w-Komanczy.jpg</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>49.347921311552</v>
       </c>
-      <c r="E6" t="n">
+      <c r="J6" t="n">
         <v>22.077292921989</v>
       </c>
     </row>
@@ -572,13 +714,36 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>620 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Smolnik 49, 38-543 Smolnik</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 40 zł </t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Schronisko-nad-Smolnikiem.jpg</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>49.280426</v>
       </c>
-      <c r="E7" t="n">
+      <c r="J7" t="n">
         <v>22.121439</v>
       </c>
     </row>
@@ -595,13 +760,36 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>650 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Stare Sioło 4, 38-608 Wetlina</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
+        <v>35</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 75 zł </t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>9,8/10</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Schronisko-Pod-Wysoka-Polonina.jpg</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>49.164366</v>
       </c>
-      <c r="E8" t="n">
+      <c r="J8" t="n">
         <v>22.457682</v>
       </c>
     </row>
@@ -618,14 +806,37 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>470 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>ul. Sobczańska 91
 34-443 Sromowce Niżne</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
+        <v>50</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 115 zł </t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-Trzy-Korony.jpg</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>49.40517</v>
       </c>
-      <c r="E9" t="n">
+      <c r="J9" t="n">
         <v>20.41125</v>
       </c>
     </row>
@@ -642,14 +853,37 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>520 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>Ul. Pienińska 12
 34-460 Szczawnica</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
+        <v>44</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 115 zł </t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Schronisko-Orlica-w-Szczawnicy.jpg</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>49.41920755404</v>
       </c>
-      <c r="E10" t="n">
+      <c r="J10" t="n">
         <v>20.457994807725</v>
       </c>
     </row>
@@ -666,13 +900,36 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>850 m n.p.m</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>Pod Homolami 4, 34-460 Jaworki</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
+        <v>50</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 45 zł </t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Schronisko-pod-Durbaszka.jpg</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>49.390816581152</v>
       </c>
-      <c r="E11" t="n">
+      <c r="J11" t="n">
         <v>20.535878865298</v>
       </c>
     </row>
@@ -689,13 +946,36 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>843 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>Języki 22, 34-460 Szczawnica.</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
+        <v>41</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 60 zł </t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>9,6/10</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Bacowka-PTTK-pod-Beresnikiem.jpg</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>49.439122285433</v>
       </c>
-      <c r="E12" t="n">
+      <c r="J12" t="n">
         <v>20.485754413756</v>
       </c>
     </row>
@@ -712,13 +992,36 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>476 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>Huta Polańska 1, Huta Polańska, 38-232 Krempna</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
+        <v>42</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 20 zł </t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>9,6/10</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>schronisko-hajstra-w-hucie-polanskiej.jpg</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>49.454746613956</v>
       </c>
-      <c r="E13" t="n">
+      <c r="J13" t="n">
         <v>21.537574297533</v>
       </c>
     </row>
@@ -735,13 +1038,36 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>655 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>Bartne 60, 38-307</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
+        <v>28</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 60 zł </t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>8,2/10</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Bacowka-PTTK-w-Bartnem.jpg</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>49.548536967276</v>
       </c>
-      <c r="E14" t="n">
+      <c r="J14" t="n">
         <v>21.357166907451</v>
       </c>
     </row>
@@ -758,13 +1084,36 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>844 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>Rytro 64, 33-343 Sucha Struga</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
+        <v>38</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 45 zł </t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>9,6/10</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Chata-Gorska-Cyrla.jpg</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>49.492123</v>
       </c>
-      <c r="E15" t="n">
+      <c r="J15" t="n">
         <v>20.716047</v>
       </c>
     </row>
@@ -781,13 +1130,36 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>887 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>33-350 Piwniczna-Zdrój</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
+        <v>40</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>od 82,5 zł</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Bacowka-PTTK-nad-Wierchomla.jpg</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>49.412547745</v>
       </c>
-      <c r="E16" t="n">
+      <c r="J16" t="n">
         <v>20.765835115</v>
       </c>
     </row>
@@ -804,14 +1176,37 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>1050 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>Schronisko Górskie PTTK na Jaworzynie Krynickiej
 33-380 Krynica-Zdrój</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="n">
+        <v>50</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 90 zł </t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Jaworzynie-Krynickiej.jpg</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>49.4215871</v>
       </c>
-      <c r="E17" t="n">
+      <c r="J17" t="n">
         <v>20.960218</v>
       </c>
     </row>
@@ -828,14 +1223,37 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>1138 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>Schronisko PTTK na Przehybie
 33-388 Gołkowice</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
+        <v>50</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 30 zł </t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>8,8/10</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Przehybie.jpg</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>49.5135502</v>
       </c>
-      <c r="E18" t="n">
+      <c r="J18" t="n">
         <v>20.5651109</v>
       </c>
     </row>
@@ -852,13 +1270,36 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>931 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>Obidza 17, 33-350 Piwniczna-Zdrój</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
+        <v>30</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 45 zł </t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Bacowka-na-Obidzy.jpg</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>49.421523683435</v>
       </c>
-      <c r="E19" t="n">
+      <c r="J19" t="n">
         <v>20.623959256627</v>
       </c>
     </row>
@@ -875,14 +1316,37 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>852 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>Bacówka PTTK na Maciejowej
 34-700 Rabka Zdrój</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="n">
+        <v>30</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 85 zł </t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-Bacowka-na-Maciejowej.jpg</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>49.5949027</v>
       </c>
-      <c r="E20" t="n">
+      <c r="J20" t="n">
         <v>19.9732606</v>
       </c>
     </row>
@@ -899,13 +1363,36 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>730 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>Sucha Działy 948, 32-432 Pcim</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="n">
+        <v>37</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 70 zł </t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>8,3/10</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Kudlaczach.jpg</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>49.7576049</v>
       </c>
-      <c r="E21" t="n">
+      <c r="J21" t="n">
         <v>19.9902211</v>
       </c>
     </row>
@@ -922,13 +1409,36 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>900 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>34-400 Nowy Targ</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="n">
+        <v>26</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 35 zł </t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Schronisko-Koliba-na-Lapsowej-Polanie.jpg</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>49.481533</v>
       </c>
-      <c r="E22" t="n">
+      <c r="J22" t="n">
         <v>20.0457527</v>
       </c>
     </row>
@@ -945,13 +1455,36 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>1022 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
           <t>Schronisko PTTK na Luboniu Wielkim 34 - 701 Rabka Zaryte 165</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
+        <v>25</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>od 50 zł</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>8,8/10</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Luboniu-Wielkim.jpg</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>49.627370281</v>
       </c>
-      <c r="E23" t="n">
+      <c r="J23" t="n">
         <v>19.987018955</v>
       </c>
     </row>
@@ -968,13 +1501,36 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
+          <t>968 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>Klikuszowa, Gorce</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="E24" t="n">
+        <v>35</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 80 zł </t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Starych-Wierchach.jpg</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>49.56024</v>
       </c>
-      <c r="E24" t="n">
+      <c r="J24" t="n">
         <v>20.03943</v>
       </c>
     </row>
@@ -990,16 +1546,39 @@
         </is>
       </c>
       <c r="C25" t="inlineStr">
+        <is>
+          <t>1283 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>Schronisko PTTK im. Władysława Orkana na Turbaczu,
 34-400 Nowy Targ
 skr. pocztowa 102</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="E25" t="n">
+        <v>110</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>od 100 zł</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Turbaczu.jpg</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>49.48581</v>
       </c>
-      <c r="E25" t="n">
+      <c r="J25" t="n">
         <v>20.03207</v>
       </c>
     </row>
@@ -1015,6 +1594,11 @@
         </is>
       </c>
       <c r="C26" t="inlineStr">
+        <is>
+          <t>1025 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
         <is>
           <t xml:space="preserve">Bacówka PTTK na Krawcowym Wierchu,
 Glinka,
@@ -1022,10 +1606,28 @@
 </t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="E26" t="n">
+        <v>29</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>od 30 zł</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Bacowka-PTTK-na-Krawcowym-Wierchu.jpg</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>49.4712</v>
       </c>
-      <c r="E26" t="n">
+      <c r="J26" t="n">
         <v>19.11847</v>
       </c>
     </row>
@@ -1042,13 +1644,36 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>1120 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>Soblówka 450, 34-371 Ujsoły</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="E27" t="n">
+        <v>34</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>od 80 zł</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Bacowka-PTTK-na-Rycerzowej.jpg</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>49.418886108053</v>
       </c>
-      <c r="E27" t="n">
+      <c r="J27" t="n">
         <v>19.097471106377</v>
       </c>
     </row>
@@ -1065,13 +1690,36 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>854 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>Boracza 23, 34-350 Żbanica</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="E28" t="n">
+        <v>35</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>od 80 zł</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Hali-Boraczej.jpg</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>49.5421</v>
       </c>
-      <c r="E28" t="n">
+      <c r="J28" t="n">
         <v>19.17061</v>
       </c>
     </row>
@@ -1088,13 +1736,36 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>1324 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>Złatna 450, 34-371 Ujsoły</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="E29" t="n">
+        <v>48</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>od 120 zł</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Hali-Lipowskiej.jpg</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>49.504291616122</v>
       </c>
-      <c r="E29" t="n">
+      <c r="J29" t="n">
         <v>19.192161446113</v>
       </c>
     </row>
@@ -1111,13 +1782,36 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>1330 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
           <t>34-335 Krzyżowa</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="E30" t="n">
+        <v>90</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>od 75 zł</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>8,8/10</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Hali-Miziowej.jpg</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>49.6008</v>
       </c>
-      <c r="E30" t="n">
+      <c r="J30" t="n">
         <v>19.3331</v>
       </c>
     </row>
@@ -1134,13 +1828,36 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
+          <t>1152 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
           <t>34-236 Sidzina</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="E31" t="n">
+        <v>38</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>od 70 zł</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>8,2/10</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Hali-Krupowej.jpg</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>49.6117</v>
       </c>
-      <c r="E31" t="n">
+      <c r="J31" t="n">
         <v>19.7294</v>
       </c>
     </row>
@@ -1157,13 +1874,34 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
+          <t>1290 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
           <t>34-371 Złatna</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="E32" t="n">
+        <v>50</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>od 70 zł</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Hali-Rysiance.jpg</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>49.4951</v>
       </c>
-      <c r="E32" t="n">
+      <c r="J32" t="n">
         <v>19.1767</v>
       </c>
     </row>
@@ -1180,13 +1918,36 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
+          <t>1180 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
           <t>34-222 Zawoja</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="E33" t="n">
+        <v>70</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>od 80 zł</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>8,6/10</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Markowych-Szczawinach.jpg</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>49.58736</v>
       </c>
-      <c r="E33" t="n">
+      <c r="J33" t="n">
         <v>19.51723</v>
       </c>
     </row>
@@ -1203,14 +1964,33 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
+          <t>1000 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
           <t>34-370 Rajcza
 Rycerk Górna 401</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="E34" t="n">
+        <v>38</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Przeleczy-Przegibek.jpg</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>49.42173</v>
       </c>
-      <c r="E34" t="n">
+      <c r="J34" t="n">
         <v>19.04766</v>
       </c>
     </row>
@@ -1227,13 +2007,36 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
+          <t>1236 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
           <t>Schronisko PTTK Wielka Racza, 34-370 Rycerka Górna</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="E35" t="n">
+        <v>46</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>od 80 zł</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>8,8/10</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Wielkiej-Raczy.jpg</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>49.4741</v>
       </c>
-      <c r="E35" t="n">
+      <c r="J35" t="n">
         <v>19.0498</v>
       </c>
     </row>
@@ -1250,13 +2053,34 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
+          <t>850 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
           <t>48-267 Jarnołtówek 211</t>
         </is>
       </c>
-      <c r="D36" t="n">
+      <c r="E36" t="n">
+        <v>50</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>od 90 zł</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-Pod-Kopa-Biskupia.jpg</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>50.260585970367</v>
       </c>
-      <c r="E36" t="n">
+      <c r="J36" t="n">
         <v>17.431095781471</v>
       </c>
     </row>
@@ -1273,13 +2097,36 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
+          <t>1500 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
           <t>Hala Gąsienicowa, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="E37" t="n">
+        <v>120</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>od 110 zł</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>8,6/10</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-Murowaniec.jpg</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>49.243322</v>
       </c>
-      <c r="E37" t="n">
+      <c r="J37" t="n">
         <v>20.007537</v>
       </c>
     </row>
@@ -1296,13 +2143,34 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
+          <t>1198 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>Droga Brata Adalberta 3, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="E38" t="n">
+        <v>96</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>od 140 zł</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Hotel-Gorski-PTTK-Kalatowki.jpg</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
         <v>49.259691806165</v>
       </c>
-      <c r="E38" t="n">
+      <c r="J38" t="n">
         <v>19.966769181176</v>
       </c>
     </row>
@@ -1319,13 +2187,36 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
+          <t>1333 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
           <t>Droga Brata Adalberta 4, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="E39" t="n">
+        <v>24</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>od 140 zł</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Hali-Kondratowej.jpg</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
         <v>49.249820313067</v>
       </c>
-      <c r="E39" t="n">
+      <c r="J39" t="n">
         <v>19.951776219509</v>
       </c>
     </row>
@@ -1342,13 +2233,36 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
+          <t>1100 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
           <t>Dolina Kościeliska 34, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="E40" t="n">
+        <v>48</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>od 130 zł</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Hali-Ornak.jpg</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
         <v>49.292859709492</v>
       </c>
-      <c r="E40" t="n">
+      <c r="J40" t="n">
         <v>19.940654607462</v>
       </c>
     </row>
@@ -1365,13 +2279,36 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
+          <t>1671 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
           <t>Schronisko Górskie PTTK w Dolinie Pięciu Stawów Polskich, 34-530 Bukowina Tatrzańska</t>
         </is>
       </c>
-      <c r="D41" t="n">
+      <c r="E41" t="n">
+        <v>67</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>od 120 zł</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>9,6/10</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-w-Dolinie-Pieciu-Stawow-Polskich.jpg</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
         <v>49.3419871</v>
       </c>
-      <c r="E41" t="n">
+      <c r="J41" t="n">
         <v>20.1038829</v>
       </c>
     </row>
@@ -1388,13 +2325,34 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
+          <t>1410 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
           <t>Schronisko Morskie Oko w Tatrach, Skrytka pocztowa 201, 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="E42" t="n">
+        <v>77</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>od 90 zł</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-nad-Morskim-Okiem.jpg</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
         <v>49.2991711</v>
       </c>
-      <c r="E42" t="n">
+      <c r="J42" t="n">
         <v>19.9490216</v>
       </c>
     </row>
@@ -1411,13 +2369,36 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
+          <t>1031 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
           <t>Schronisko PTTK w Dolinie Roztoki Skrytka pocztowa 200 34-500 Zakopane</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="E43" t="n">
+        <v>70</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>od 100 zł</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>9,8/10</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-w-Dolinie-Roztoki.jpg</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>49.2991711</v>
       </c>
-      <c r="E43" t="n">
+      <c r="J43" t="n">
         <v>19.9490216</v>
       </c>
     </row>
@@ -1434,13 +2415,36 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
+          <t>1120 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
           <t>DW960 10, Głodówka 20, 34-532 Brzegi</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="E44" t="n">
+        <v>90</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>od 70 zł</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Schronisko-GK-ZHP-Glodowka.jpg</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>49.301997031691</v>
       </c>
-      <c r="E44" t="n">
+      <c r="J44" t="n">
         <v>20.11679024441</v>
       </c>
     </row>
@@ -1457,13 +2461,36 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
+          <t>1146 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
           <t>Witów N, 34-512 Dolina Chochołowska</t>
         </is>
       </c>
-      <c r="D45" t="n">
+      <c r="E45" t="n">
+        <v>121</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>od 80 zł</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Polanie-Chocholowskiej.jpg</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
         <v>49.2363</v>
       </c>
-      <c r="E45" t="n">
+      <c r="J45" t="n">
         <v>19.7878</v>
       </c>
     </row>
@@ -1480,13 +2507,34 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
+          <t>890 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
           <t>Schronisko PTTK "LESKOWIEC", 34-206 Krzeszów</t>
         </is>
       </c>
-      <c r="D46" t="n">
+      <c r="E46" t="n">
+        <v>32</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>od 75 zł</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-Leskowiec.jpg</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
         <v>49.7592</v>
       </c>
-      <c r="E46" t="n">
+      <c r="J46" t="n">
         <v>19.4885</v>
       </c>
     </row>
@@ -1503,13 +2551,36 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
+          <t>90 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
           <t>Magurka Wilkowicka 7, 43-365 Wilkowice</t>
         </is>
       </c>
-      <c r="D47" t="n">
+      <c r="E47" t="n">
+        <v>24</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>od 140 zł</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>8,8/10</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Magurce-Wilkowickiej.jpg</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
         <v>49.776611</v>
       </c>
-      <c r="E47" t="n">
+      <c r="J47" t="n">
         <v>19.1300746</v>
       </c>
     </row>
@@ -1526,13 +2597,36 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
+          <t>685 m n.p.m</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
           <t>adres biura: SST Rogacz Sp. z o.o. ul. Wyzwolenia 30 41-600 Świętochłowice</t>
         </is>
       </c>
-      <c r="D48" t="n">
+      <c r="E48" t="n">
+        <v>40</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 40 zł </t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>schronisko-na-rogaczu.jpg</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
         <v>50.291769793393</v>
       </c>
-      <c r="E48" t="n">
+      <c r="J48" t="n">
         <v>18.920813444499</v>
       </c>
     </row>
@@ -1549,13 +2643,32 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
+          <t>820 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
           <t>Schronisko na Iglicznej koło Międzygórza Góra Igliczna, 57-500 600 215 170</t>
         </is>
       </c>
-      <c r="D49" t="n">
+      <c r="E49" t="n">
+        <v>40</v>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>6,8/10</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Schronisko-na-Iglicznej.jpg</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>21.50951</v>
       </c>
-      <c r="E49" t="n">
+      <c r="J49" t="n">
         <v>-104.89569</v>
       </c>
     </row>
@@ -1572,13 +2685,36 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
+          <t>1218 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
           <t>Schronisko PTTK Na Śnieżniku Międzygórze 57-514 Międzygórze</t>
         </is>
       </c>
-      <c r="D50" t="n">
+      <c r="E50" t="n">
+        <v>48</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>od 80 zł</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>8,4/10</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-na-sniezniku.jpg</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
         <v>50.223857908146</v>
       </c>
-      <c r="E50" t="n">
+      <c r="J50" t="n">
         <v>16.774280907033</v>
       </c>
     </row>
@@ -1595,13 +2731,34 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
+          <t>1117 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
           <t>Schronisko Górskie PTTK "KLIMCZOK" Dorota Kukla,Natalia Kukla,Piotr Kukla S.C. 43-309 Bielsko-Biała</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="E51" t="n">
+        <v>38</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>od 90 zł</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-Klimczok.jpg</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
         <v>49.7794751</v>
       </c>
-      <c r="E51" t="n">
+      <c r="J51" t="n">
         <v>19.0510662</v>
       </c>
     </row>
@@ -1618,13 +2775,36 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
+          <t>951 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
           <t>Schronisko PTTK Przysłop pod Baranią Górą Czarna Wisełka 8 43-460 Wisła</t>
         </is>
       </c>
-      <c r="D52" t="n">
+      <c r="E52" t="n">
+        <v>50</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>od 90 zł</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Schronisko-na-Przyslopie-pod-PPTK-Barania-Gore.jpg</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
         <v>49.596287160924</v>
       </c>
-      <c r="E52" t="n">
+      <c r="J52" t="n">
         <v>18.983642849598</v>
       </c>
     </row>
@@ -1641,13 +2821,34 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
+          <t>758 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
           <t>Ustroń, 43 -450 ul. Równica 27</t>
         </is>
       </c>
-      <c r="D53" t="n">
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 159 zł </t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>8,4/10</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-na-rownicy.jpg</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
         <v>49.719607713502</v>
       </c>
-      <c r="E53" t="n">
+      <c r="J53" t="n">
         <v>18.851971281158</v>
       </c>
     </row>
@@ -1664,13 +2865,34 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
+          <t>1250 m n.p.m</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
           <t>Schronisko PTTK Skrzyczne s.c. Adres: 43-370 Szczyrk</t>
         </is>
       </c>
-      <c r="D54" t="n">
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>od 100 zł</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>8,8/10</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Schronisko-Skrzyczne-w-Szczyrku.jpg</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
         <v>49.7050608</v>
       </c>
-      <c r="E54" t="n">
+      <c r="J54" t="n">
         <v>19.0065914</v>
       </c>
     </row>
@@ -1687,13 +2909,36 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
+          <t>957 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
           <t>Schronisko PTTK Stożek ul. Turystyczna 19 43-460 Wisła</t>
         </is>
       </c>
-      <c r="D55" t="n">
+      <c r="E55" t="n">
+        <v>72</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 90 zł </t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>8,6/10</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Schronisko-na-Stozku.jpg</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
         <v>49.604283412734</v>
       </c>
-      <c r="E55" t="n">
+      <c r="J55" t="n">
         <v>18.82344691028</v>
       </c>
     </row>
@@ -1710,13 +2955,36 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
+          <t>1001 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
           <t>Schronisko górskie PTTK Szyndzielnia 43 - 360 Bystra ul. Schronisko Szyndzielnia 8</t>
         </is>
       </c>
-      <c r="D56" t="n">
+      <c r="E56" t="n">
+        <v>49</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 70 zł </t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-na-szyndzielni.jpg</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
         <v>49.7658456</v>
       </c>
-      <c r="E56" t="n">
+      <c r="J56" t="n">
         <v>19.0737288</v>
       </c>
     </row>
@@ -1733,13 +3001,36 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
+          <t>891 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
           <t>Schronisko PTTK na Błatniej Adres 43-438 Brenna, ul. Błatnia 20</t>
         </is>
       </c>
-      <c r="D57" t="n">
+      <c r="E57" t="n">
+        <v>49</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 90 zł </t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-na-blatniej.jpg</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
         <v>49.747</v>
       </c>
-      <c r="E57" t="n">
+      <c r="J57" t="n">
         <v>18.94215</v>
       </c>
     </row>
@@ -1756,13 +3047,32 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
+          <t>715 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
           <t>Chata Wuja Toma Przełęcz Karkoszczonka ul. Pasterska 9 43-370 Szczyrk</t>
         </is>
       </c>
-      <c r="D58" t="n">
+      <c r="E58" t="n">
+        <v>40</v>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>schronisko-chata-wuja-toma.jpg</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
         <v>49.725339803717</v>
       </c>
-      <c r="E58" t="n">
+      <c r="J58" t="n">
         <v>18.993476079308</v>
       </c>
     </row>
@@ -1779,13 +3089,34 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
+          <t>676 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
           <t>ul. Pocztowa 34 43-309 Bielsko-Biała</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="E59" t="n">
+        <v>30</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>od 140 zł</t>
+        </is>
+      </c>
+      <c r="G59" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>schronisko-na-koziej-gorze.jpg</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
         <v>49.768060017269</v>
       </c>
-      <c r="E59" t="n">
+      <c r="J59" t="n">
         <v>19.039150410816</v>
       </c>
     </row>
@@ -1802,13 +3133,36 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
+          <t>520 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
           <t>GOSPODA DĘBOWIEC 520 Skalna 90, 43-309 Bielsko-Biała</t>
         </is>
       </c>
-      <c r="D60" t="n">
+      <c r="E60" t="n">
+        <v>11</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 150 zł </t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>8,6/10</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>schronisko-na-debowcu.jpg</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
         <v>49.7804</v>
       </c>
-      <c r="E60" t="n">
+      <c r="J60" t="n">
         <v>19.015</v>
       </c>
     </row>
@@ -1825,13 +3179,36 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
+          <t>799 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
           <t>Soszowska 10, 43-460 Wisła</t>
         </is>
       </c>
-      <c r="D61" t="n">
+      <c r="E61" t="n">
+        <v>30</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>od 80 zł</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>schronisko-na-soszowie-wielkim.jpg</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
         <v>49.6392923</v>
       </c>
-      <c r="E61" t="n">
+      <c r="J61" t="n">
         <v>18.8138184</v>
       </c>
     </row>
@@ -1848,13 +3225,32 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
+          <t>810 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
           <t>ul. Pilarzy 64 43-438 Brenna</t>
         </is>
       </c>
-      <c r="D62" t="n">
+      <c r="E62" t="n">
+        <v>25</v>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Schronisko--Telesforowka-na-Trzech-Kopcach-Wislanskich.jpg</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
         <v>49.665096802481</v>
       </c>
-      <c r="E62" t="n">
+      <c r="J62" t="n">
         <v>18.90752779269</v>
       </c>
     </row>
@@ -1871,13 +3267,34 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
+          <t>875 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
           <t>Schronisko Górskie „Orzeł” Sokolec 52 57-450 Ludwikowice Kłodzkie</t>
         </is>
       </c>
-      <c r="D63" t="n">
+      <c r="E63" t="n">
+        <v>92</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 55 zł </t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Schronisko-Orzel.jpg</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
         <v>50.6642</v>
       </c>
-      <c r="E63" t="n">
+      <c r="J63" t="n">
         <v>16.4732</v>
       </c>
     </row>
@@ -1894,13 +3311,34 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
+          <t>740 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
           <t>Schronisko PTTK "Zygmuntówka" im. Zygmunta Scheffnera 57-430 Jugów, ul. Świętojańska 30</t>
         </is>
       </c>
-      <c r="D64" t="n">
+      <c r="E64" t="n">
+        <v>31</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 75 zł </t>
+        </is>
+      </c>
+      <c r="G64" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-zygmuntowka.jpg</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
         <v>50.645982419546</v>
       </c>
-      <c r="E64" t="n">
+      <c r="J64" t="n">
         <v>16.516789503312</v>
       </c>
     </row>
@@ -1917,13 +3355,36 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
+          <t>480 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
           <t>Jamna 14 32-842 Paleśnica woj. małopolskie Polska</t>
         </is>
       </c>
-      <c r="D65" t="n">
+      <c r="E65" t="n">
+        <v>80</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 50 zł </t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>8,6/10</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Bacowka-na-Jamnej.jpg</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
         <v>49.769800896649</v>
       </c>
-      <c r="E65" t="n">
+      <c r="J65" t="n">
         <v>20.831419239208</v>
       </c>
     </row>
@@ -1938,15 +3399,34 @@
           <t>Pogórze Ciężkowickie</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
         <is>
           <t>Jamna 46, 32-842 Jamna</t>
         </is>
       </c>
-      <c r="D66" t="n">
+      <c r="E66" t="n">
+        <v>30</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 85 zł </t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>9,6/10</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>chata-wloczykija.jpg</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
         <v>49.768355940361</v>
       </c>
-      <c r="E66" t="n">
+      <c r="J66" t="n">
         <v>20.83027033174</v>
       </c>
     </row>
@@ -1961,15 +3441,34 @@
           <t>Pogórze Ciężkowickie</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
         <is>
           <t>Schronisko Dobrych Myśli Jamna 53, 32-842 Jamna Małopolska</t>
         </is>
       </c>
-      <c r="D67" t="n">
+      <c r="E67" t="n">
+        <v>15</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>od 85 zł</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>schronisko-dobrych-mysli.jpg</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
         <v>49.76819672611</v>
       </c>
-      <c r="E67" t="n">
+      <c r="J67" t="n">
         <v>20.830788920089</v>
       </c>
     </row>
@@ -1986,13 +3485,36 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
+          <t>320 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
           <t>Gościniec Perła Zachodu 58-522 Siedlęcin 1</t>
         </is>
       </c>
-      <c r="D68" t="n">
+      <c r="E68" t="n">
+        <v>14</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 150 zł </t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>8.8/10</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>schronisko-perla-zachodu.jpg</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
         <v>50.928153435847</v>
       </c>
-      <c r="E68" t="n">
+      <c r="J68" t="n">
         <v>15.69125997445</v>
       </c>
     </row>
@@ -2009,13 +3531,30 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
+          <t>718 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
           <t>DOM TURYSTY im. Romana Zmorskiego Góra Ślęża 55-050 Sobótka woj. Dolnośląskie</t>
         </is>
       </c>
-      <c r="D69" t="n">
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>7,6/10</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-na-slezy.jpg</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
         <v>50.900072</v>
       </c>
-      <c r="E69" t="n">
+      <c r="J69" t="n">
         <v>16.743953</v>
       </c>
     </row>
@@ -2032,220 +3571,1032 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
+          <t>280 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
           <t>ul. Armii Krajowej 13 55-050 Sobótka</t>
         </is>
       </c>
-      <c r="D70" t="n">
+      <c r="E70" t="n">
+        <v>50</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>od 70 zł</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>8,8/10</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>dom-turysty-pttk-pod-wiezyca.jpg</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
         <v>50.892757992676</v>
       </c>
-      <c r="E70" t="n">
+      <c r="J70" t="n">
         <v>16.726494811814</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Schronisko "Kamieńczyk"</t>
+          <t>Schronisko PTTK "Orlica" w Zieleńcu</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Karkonosze</t>
+          <t>Góry Orlickie</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ul. Jedności Narodowej 1A</t>
-        </is>
-      </c>
-      <c r="D71" t="n">
-        <v>50.814342898</v>
+          <t>850 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Zieleniec 78, 57-340 Duszniki-Zdrój</t>
+        </is>
       </c>
       <c r="E71" t="n">
-        <v>15.496669854</v>
+        <v>25</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>od 75 zł</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>8,6/10</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-orlica.jpg</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>50.340278046364</v>
+      </c>
+      <c r="J71" t="n">
+        <v>16.384615170017</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Schronisko PTTK "Kochanówka"</t>
+          <t>Schronisko PTTK "Na Szczelińcu"</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Karkonosze</t>
+          <t>Góry Stołowe</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>58-573 Piechowice</t>
-        </is>
-      </c>
-      <c r="D72" t="n">
-        <v>50.830093</v>
+          <t>905 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Karłów 9, 57-350 Kudowa Zdrój</t>
+        </is>
       </c>
       <c r="E72" t="n">
-        <v>15.555366</v>
+        <v>30</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>od 80 zł</t>
+        </is>
+      </c>
+      <c r="G72" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-na-szczelincu.jpg</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>50.4855</v>
+      </c>
+      <c r="J72" t="n">
+        <v>16.3395</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Schronisko PTTK "Odrodzenie" na Przełęczy Karkonoskiej</t>
+          <t>Schronisko PTTK "Pasterka"</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Karkonosze</t>
+          <t>Góry Stołowe</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Karkonoska 1, 58-563 Przesieka</t>
-        </is>
-      </c>
-      <c r="D73" t="n">
-        <v>50.81219</v>
+          <t>700 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Pasterka 18, 57-350 Kudowa-Zdrój</t>
+        </is>
       </c>
       <c r="E73" t="n">
-        <v>15.67468</v>
+        <v>49</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>od 70 zł</t>
+        </is>
+      </c>
+      <c r="G73" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-pasterka.jpg</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>50.495277</v>
+      </c>
+      <c r="J73" t="n">
+        <v>16.327132</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Schronisko PTTK "Pod Łabskim Szczytem"</t>
+          <t>Schronisko PTTK na Zamku Grodno</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Karkonosze</t>
+          <t>Góry Wałbrzyskie</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Szlak pieszy żółty, 58-580 Szklarska Poręba</t>
-        </is>
-      </c>
-      <c r="D74" t="n">
-        <v>50.8301877</v>
-      </c>
-      <c r="E74" t="n">
-        <v>15.5187449</v>
+          <t>450 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Zamek Grodno, 58-321 Zagórze Śląskie</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>od 300 zł</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>schronisko-zamek-grodno.jpg</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>50.7529051</v>
+      </c>
+      <c r="J74" t="n">
+        <v>16.4054086</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Schronisko PTTK "Samotnia"</t>
+          <t xml:space="preserve">Schronisko PTTK "Jagodna" na Przełęczy Spalonej </t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Karkonosze</t>
+          <t xml:space="preserve">Góry Bystrzyckie </t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Na Śnieżkę 16, 58-550 Karpacz</t>
-        </is>
-      </c>
-      <c r="D75" t="n">
-        <v>50.749122095643</v>
+          <t>811 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Spalona 6 57-500 Bystrzyca Kłodzka</t>
+        </is>
       </c>
       <c r="E75" t="n">
-        <v>15.702750615637</v>
+        <v>57</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 40 zł </t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>9,6/10</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-jagodna.jpg</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>50.277562</v>
+      </c>
+      <c r="J75" t="n">
+        <v>16.538052</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Schronisko PTTK "Srebrny Potok" w Dolinie Srebrnika</t>
+          <t>Schronisko PTTK "Pod Muflonem"</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Karkonosze</t>
+          <t xml:space="preserve">Góry Bystrzyckie </t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Jarkowice 136, Jarkowice, Poland</t>
-        </is>
-      </c>
-      <c r="D76" t="n">
-        <v>50.7159893544</v>
+          <t>690 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Górska 14, 57-340 Duszniki-Zdrój</t>
+        </is>
       </c>
       <c r="E76" t="n">
-        <v>15.881337121074</v>
+        <v>48</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>od 37 zł</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-pod-muflonem.jpg</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>50.391574078422</v>
+      </c>
+      <c r="J76" t="n">
+        <v>16.397949353046</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Schronisko PTTK "Strzecha Akademicka"</t>
+          <t>Schronisko PTTK "Andrzejówka" na Przełęczy Trzech Dolin</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Karkonosze</t>
+          <t>Góry Kamienne</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Na Śnieżkę 18, 58-540 Karpacz</t>
-        </is>
-      </c>
-      <c r="D77" t="n">
-        <v>50.75092</v>
+          <t>780 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Rybnica Leśna 27, 58-350 Mieroszów</t>
+        </is>
       </c>
       <c r="E77" t="n">
-        <v>15.70839</v>
+        <v>38</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>od 50 zł</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>9,8/10</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-andrzejowka.jpg</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>50.684986915758</v>
+      </c>
+      <c r="J77" t="n">
+        <v>16.277975652496</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Schronisko Górskie "Dom Śląski"</t>
+          <t>Schronisko PTTK "Szwajcarka" pod Krzyżną Górą</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Karkonosze</t>
+          <t xml:space="preserve">Rudawy Janowickie </t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Na Śnieżkę 20 58-540 Karpacz</t>
-        </is>
-      </c>
-      <c r="D78" t="n">
-        <v>50.739536</v>
+          <t>520 m n.p.m</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Janowicka 7, 58-533 Karpniki</t>
+        </is>
       </c>
       <c r="E78" t="n">
-        <v>15.728889</v>
+        <v>44</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 60 zł </t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-szwajcarka.jpg</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>50.863232319645</v>
+      </c>
+      <c r="J78" t="n">
+        <v>15.872586246521</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
+          <t>Schronisko PTTK na Stogu Izerskim</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Góry Izerskie</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>1060 m n.p.m</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>ul. Nadbrzeżna 1, 59-850 Świeradów-Zdrój</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>25</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>od 180</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>8,2/10</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-na-stogu-izerskim.jpg</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>50.906774923628</v>
+      </c>
+      <c r="J79" t="n">
+        <v>15.344191740893</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Schronisko Turystyczne "Chatka Górzystów"</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Góry Izerskie</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>840 m n.p.m</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Hala Izerska 1, 59-850 Świeradów-Zdrój</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>40</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>od 30 zł</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>9,6/10</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>schronisko-turystyczne-chatka-gorzystow.jpg</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>50.918227034117</v>
+      </c>
+      <c r="J80" t="n">
+        <v>15.303095437262</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>"Schronisko Turystyczne "Orle"</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Góry Izerskie</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>840 m n.p.m</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Osiedle Orle 1, 58-580 Szklarska Poręba</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>73</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 55 zł </t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>8,8/10</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>schronisko-turystyczne-orle.jpg</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>50.815062318377</v>
+      </c>
+      <c r="J81" t="n">
+        <v>15.383251577329</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Schronisko na Hali Szrenickiej</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Karkonosze</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>1195 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Główny Szlak Sudecki 58/580, 58-580 Szklarska Poręba</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ponad 100</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>od 70 zł</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>9,2/10</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-na-hali-szrenickiej.jpg</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>50.838235652171</v>
+      </c>
+      <c r="J82" t="n">
+        <v>15.505600754446</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Schronisko na Szrenicy</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Karkonosze</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>1362 m.n.p.m.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Szrenica I, 58-580 Szklarska Poręba</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>90</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>od 106 zł za pokój</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>9,2/11</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>schronisko-na-szrenicy.jpg</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>50.79198</v>
+      </c>
+      <c r="J83" t="n">
+        <v>15.51366</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Schronisko "Kamieńczyk"</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Karkonosze</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>830 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ul. Jedności Narodowej 1A</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>19</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>od 50 zł</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>8,4/10</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>schronisko-kamienczyk.jpg</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>50.814342898</v>
+      </c>
+      <c r="J84" t="n">
+        <v>15.496669854</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Schronisko PTTK "Kochanówka"</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Karkonosze</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>510 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>58-573 Piechowice</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>12</v>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-kochanowka.jpg</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>50.830093</v>
+      </c>
+      <c r="J85" t="n">
+        <v>15.555366</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Schronisko PTTK "Odrodzenie" na Przełęczy Karkonoskiej</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Karkonosze</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>1236 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Karkonoska 1, 58-563 Przesieka</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>100</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>od 90 zł</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>8,8/10</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Schronisko-pttk-Odrodzenie.jpg</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>50.81219</v>
+      </c>
+      <c r="J86" t="n">
+        <v>15.67468</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Schronisko PTTK "Pod Łabskim Szczytem"</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Karkonosze</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>1168 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Szlak pieszy żółty, 58-580 Szklarska Poręba</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>38</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 45 zł </t>
+        </is>
+      </c>
+      <c r="G87" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-pod-labskim-szczytem.jpg</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>50.8301877</v>
+      </c>
+      <c r="J87" t="n">
+        <v>15.5187449</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Schronisko PTTK "Samotnia"</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Karkonosze</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1195 m n.p.m. </t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Na Śnieżkę 16, 58-550 Karpacz</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>49</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>od 90 zł</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-samotnia.jpg</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>50.749122095643</v>
+      </c>
+      <c r="J88" t="n">
+        <v>15.702750615637</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Schronisko PTTK "Srebrny Potok" w Dolinie Srebrnika</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Karkonosze</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>650 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Jarkowice 136, Jarkowice, Poland</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>45</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>od 35 zł</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>9,4/10</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>schronisko-pttk-srebrny-potok.jpg</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>50.7159893544</v>
+      </c>
+      <c r="J89" t="n">
+        <v>15.881337121074</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Schronisko PTTK "Strzecha Akademicka"</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Karkonosze</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>1266 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Na Śnieżkę 18, 58-540 Karpacz</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>75</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>od 150 zł</t>
+        </is>
+      </c>
+      <c r="G90" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>scronisko-pttk-strzecha-akademicka.jpg</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>50.75092</v>
+      </c>
+      <c r="J90" t="n">
+        <v>15.70839</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Schronisko Górskie "Dom Śląski"</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Karkonosze</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1400 m n.p.m. </t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Na Śnieżkę 20 58-540 Karpacz</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>58</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od 70 zł </t>
+        </is>
+      </c>
+      <c r="G91" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>schronisko-dom-slaski.jpg</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>50.739536</v>
+      </c>
+      <c r="J91" t="n">
+        <v>15.728889</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
           <t>Schronisko PTTK na Przełęczy Okraj</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>Karkonosze</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>1046 m n.p.m.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
         <is>
           <t>Schronisko PTTK, Przełęcz Okraj 1 Kowary 58-530</t>
         </is>
       </c>
-      <c r="D79" t="n">
+      <c r="E92" t="n">
+        <v>40</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>od 80 zł</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>7,8/10</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Schronisko-PTTK-na-Przeleczy-Okraj.jpg</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
         <v>50.74709</v>
       </c>
-      <c r="E79" t="n">
+      <c r="J92" t="n">
         <v>15.82411</v>
       </c>
     </row>

</xml_diff>